<commit_message>
Agregando las pruebas de confianza al informe
</commit_message>
<xml_diff>
--- a/PRUEBAS DE CONFIANZA.xlsx
+++ b/PRUEBAS DE CONFIANZA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omich\Documents\SolucionesEnergeticasParaWSN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EAB052-DE0F-49D2-8372-D89A9AA3552D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88EC254F-F5C9-4BB0-8ADB-B749F535FF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF7E538C-BC1E-4233-9CFA-651CC43E1462}"/>
   </bookViews>
@@ -19,6 +19,12 @@
     <definedName name="_xlchart.v1.0" hidden="1">(Hoja1!$C$4:$C$11,Hoja1!$C$13:$C$20,Hoja1!$C$22:$C$29)</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">(Hoja1!$H$4:$H$11,Hoja1!$H$13:$H$20,Hoja1!$H$22:$H$29)</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$H$3</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">(Hoja1!$C$4:$C$11,Hoja1!$C$13:$C$20,Hoja1!$C$22:$C$29)</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">(Hoja1!$H$4:$H$11,Hoja1!$H$13:$H$20,Hoja1!$H$22:$H$29)</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Hoja1!$H$3</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">(Hoja1!$C$4:$C$11,Hoja1!$C$13:$C$20,Hoja1!$C$22:$C$29)</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">(Hoja1!$H$4:$H$11,Hoja1!$H$13:$H$20,Hoja1!$H$22:$H$29)</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Hoja1!$H$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="27">
   <si>
     <t>SOFTWARE</t>
   </si>
@@ -122,6 +128,9 @@
   </si>
   <si>
     <t>|</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -216,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -233,6 +242,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,7 +471,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.57471264367816088</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -604,34 +614,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx2"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="es-MX"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -929,7 +911,7 @@
         <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -991,7 +973,7 @@
           </c:spPr>
         </c:majorGridlines>
         <c:numFmt formatCode="0.00" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1342,7 +1324,7 @@
         <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1404,7 +1386,7 @@
           </c:spPr>
         </c:majorGridlines>
         <c:numFmt formatCode="0.00" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1688,7 +1670,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>199</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>148</c:v>
@@ -1700,7 +1682,7 @@
                   <c:v>138</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>346</c:v>
+                  <c:v>198</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>198</c:v>
@@ -3440,10 +3422,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>199</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>199</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="2" formatCode="0.00">
                   <c:v>0</c:v>
@@ -9316,14 +9298,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>257577</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>32197</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>180047</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1894659</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>113731</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>160985</xdr:rowOff>
+      <xdr:rowOff>170596</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9353,13 +9335,13 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>683079</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>8560</xdr:rowOff>
+      <xdr:rowOff>8559</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>246323</xdr:colOff>
+      <xdr:colOff>227463</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>146406</xdr:rowOff>
+      <xdr:rowOff>170596</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9998,7 +9980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC5ECB90-EE67-49F2-B71E-283C8DA9AB5B}">
-  <dimension ref="A3:L71"/>
+  <dimension ref="A3:M71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" customWidth="1"/>
@@ -10007,11 +9989,11 @@
     <col min="5" max="5" width="25.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.109375" customWidth="1"/>
-    <col min="11" max="11" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:12" ht="18" x14ac:dyDescent="0.35">
@@ -10066,10 +10048,10 @@
         <v>15</v>
       </c>
       <c r="E4" s="1">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F4" s="1">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G4" s="1">
         <f>E4-F4</f>
@@ -10085,11 +10067,11 @@
       </c>
       <c r="J4" s="1">
         <f>F4/10</f>
-        <v>19.899999999999999</v>
+        <v>20</v>
       </c>
       <c r="K4" s="5">
         <f>F4 / 600</f>
-        <v>0.33166666666666667</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="L4" s="10">
         <f>F4/E4</f>
@@ -10242,10 +10224,10 @@
         <v>15</v>
       </c>
       <c r="E8" s="1">
-        <v>348</v>
+        <v>200</v>
       </c>
       <c r="F8" s="1">
-        <v>346</v>
+        <v>198</v>
       </c>
       <c r="G8" s="1">
         <f t="shared" si="0"/>
@@ -10253,23 +10235,23 @@
       </c>
       <c r="H8" s="5">
         <f t="shared" si="1"/>
-        <v>0.57471264367816088</v>
+        <v>1</v>
       </c>
       <c r="I8" s="5">
         <f t="shared" si="2"/>
-        <v>99.425287356321846</v>
+        <v>99</v>
       </c>
       <c r="J8" s="1">
         <f t="shared" si="3"/>
-        <v>34.6</v>
+        <v>19.8</v>
       </c>
       <c r="K8" s="5">
         <f t="shared" si="4"/>
-        <v>0.57666666666666666</v>
+        <v>0.33</v>
       </c>
       <c r="L8" s="10">
         <f t="shared" si="5"/>
-        <v>0.99425287356321834</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -10380,7 +10362,7 @@
         <v>200</v>
       </c>
       <c r="G11" s="1">
-        <f t="shared" si="0"/>
+        <f>E11-F11</f>
         <v>0</v>
       </c>
       <c r="H11" s="5">
@@ -10752,7 +10734,7 @@
         <v>200</v>
       </c>
       <c r="G20" s="2">
-        <f t="shared" si="0"/>
+        <f>E20-F20</f>
         <v>8</v>
       </c>
       <c r="H20" s="6">
@@ -11146,6 +11128,19 @@
       <c r="L29" s="7">
         <f t="shared" si="5"/>
         <v>0.995</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K30" s="12"/>
+    </row>
+    <row r="47" spans="12:13" x14ac:dyDescent="0.3">
+      <c r="M47" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="12:13" x14ac:dyDescent="0.3">
+      <c r="L48" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.3">

</xml_diff>